<commit_message>
Fix PPT report generation, align with website dashboard KPIs and financials, and add Vercel config
</commit_message>
<xml_diff>
--- a/excel_template/GrayQuest_Mastersheet_Template.xlsx
+++ b/excel_template/GrayQuest_Mastersheet_Template.xlsx
@@ -19,10 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -136,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -176,11 +175,14 @@
     <xf numFmtId="3" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -724,85 +726,85 @@
         </is>
       </c>
       <c r="B1" s="13" t="n">
-        <v>45412</v>
+        <v>45383.5</v>
       </c>
       <c r="C1" s="13" t="n">
-        <v>45443</v>
+        <v>45413.5</v>
       </c>
       <c r="D1" s="13" t="n">
-        <v>45473</v>
+        <v>45444.5</v>
       </c>
       <c r="E1" s="13" t="n">
-        <v>45504</v>
+        <v>45474.5</v>
       </c>
       <c r="F1" s="13" t="n">
-        <v>45535</v>
+        <v>45505.5</v>
       </c>
       <c r="G1" s="13" t="n">
-        <v>45565</v>
+        <v>45536.5</v>
       </c>
       <c r="H1" s="13" t="n">
-        <v>45566</v>
+        <v>45566.5</v>
       </c>
       <c r="I1" s="13" t="n">
-        <v>45626</v>
+        <v>45597.5</v>
       </c>
       <c r="J1" s="13" t="n">
-        <v>45657</v>
+        <v>45627.5</v>
       </c>
       <c r="K1" s="13" t="n">
-        <v>45688</v>
+        <v>45658.5</v>
       </c>
       <c r="L1" s="13" t="n">
-        <v>45716</v>
+        <v>45689.5</v>
       </c>
       <c r="M1" s="13" t="n">
-        <v>45747</v>
+        <v>45717.5</v>
       </c>
       <c r="N1" s="13" t="n">
-        <v>45777</v>
+        <v>45748.5</v>
       </c>
       <c r="O1" s="13" t="n">
-        <v>45808</v>
+        <v>45778.5</v>
       </c>
       <c r="P1" s="13" t="n">
-        <v>45838</v>
+        <v>45809.5</v>
       </c>
       <c r="Q1" s="13" t="n">
-        <v>45869</v>
+        <v>45839.5</v>
       </c>
       <c r="R1" s="13" t="n">
-        <v>45900</v>
+        <v>45870.5</v>
       </c>
       <c r="S1" s="13" t="n">
-        <v>45930</v>
+        <v>45901.5</v>
       </c>
       <c r="T1" s="13" t="n">
-        <v>45961</v>
+        <v>45931.5</v>
       </c>
       <c r="U1" s="13" t="n">
-        <v>45991</v>
+        <v>45962.5</v>
       </c>
       <c r="V1" s="13" t="n">
-        <v>46022</v>
+        <v>45992.5</v>
       </c>
       <c r="W1" s="13" t="n">
-        <v>46053</v>
+        <v>46023.5</v>
       </c>
       <c r="X1" s="13" t="n">
-        <v>46081</v>
+        <v>46054.5</v>
       </c>
       <c r="Y1" s="13" t="n">
-        <v>46112</v>
+        <v>46082.5</v>
       </c>
       <c r="Z1" s="13" t="n">
-        <v>46142</v>
+        <v>46113.5</v>
       </c>
       <c r="AA1" s="13" t="n">
-        <v>46173</v>
+        <v>46143.5</v>
       </c>
       <c r="AB1" s="13" t="n">
-        <v>46203</v>
+        <v>46174.5</v>
       </c>
     </row>
     <row r="2">
@@ -1939,85 +1941,85 @@
           <t>Average Loan IRR</t>
         </is>
       </c>
-      <c r="B17" s="17" t="n">
+      <c r="B17" s="20" t="n">
         <v>0.1901</v>
       </c>
-      <c r="C17" s="17" t="n">
+      <c r="C17" s="20" t="n">
         <v>0.2265</v>
       </c>
-      <c r="D17" s="17" t="n">
+      <c r="D17" s="20" t="n">
         <v>0.2136</v>
       </c>
-      <c r="E17" s="17" t="n">
+      <c r="E17" s="20" t="n">
         <v>0.221</v>
       </c>
-      <c r="F17" s="17" t="n">
+      <c r="F17" s="20" t="n">
         <v>0.232</v>
       </c>
-      <c r="G17" s="17" t="n">
+      <c r="G17" s="20" t="n">
         <v>0.233</v>
       </c>
-      <c r="H17" s="17" t="n">
+      <c r="H17" s="20" t="n">
         <v>0.224</v>
       </c>
-      <c r="I17" s="17" t="n">
+      <c r="I17" s="20" t="n">
         <v>0.2304</v>
       </c>
-      <c r="J17" s="17" t="n">
+      <c r="J17" s="20" t="n">
         <v>0.2346</v>
       </c>
-      <c r="K17" s="17" t="n">
+      <c r="K17" s="20" t="n">
         <v>0.2152</v>
       </c>
-      <c r="L17" s="17" t="n">
+      <c r="L17" s="20" t="n">
         <v>0.1957</v>
       </c>
-      <c r="M17" s="17" t="n">
+      <c r="M17" s="20" t="n">
         <v>0.192</v>
       </c>
-      <c r="N17" s="17" t="n">
+      <c r="N17" s="20" t="n">
         <v>0.1912</v>
       </c>
-      <c r="O17" s="17" t="n">
+      <c r="O17" s="20" t="n">
         <v>0.2168</v>
       </c>
-      <c r="P17" s="17" t="n">
+      <c r="P17" s="20" t="n">
         <v>0.2119</v>
       </c>
-      <c r="Q17" s="17" t="n">
+      <c r="Q17" s="20" t="n">
         <v>0.2142</v>
       </c>
-      <c r="R17" s="17" t="n">
+      <c r="R17" s="20" t="n">
         <v>0.2373</v>
       </c>
-      <c r="S17" s="17" t="n">
+      <c r="S17" s="20" t="n">
         <v>0.2337</v>
       </c>
-      <c r="T17" s="17" t="n">
+      <c r="T17" s="20" t="n">
         <v>0.2531</v>
       </c>
-      <c r="U17" s="17" t="n">
+      <c r="U17" s="20" t="n">
         <v>0.2406</v>
       </c>
-      <c r="V17" s="17" t="n">
+      <c r="V17" s="20" t="n">
         <v>0.2151</v>
       </c>
-      <c r="W17" s="17" t="n">
+      <c r="W17" s="20" t="n">
         <v>0.2151</v>
       </c>
-      <c r="X17" s="17" t="n">
+      <c r="X17" s="20" t="n">
         <v>0.1998</v>
       </c>
-      <c r="Y17" s="17" t="n">
+      <c r="Y17" s="20" t="n">
         <v>0.1876</v>
       </c>
-      <c r="Z17" s="17" t="n">
+      <c r="Z17" s="20" t="n">
         <v>0.1841</v>
       </c>
-      <c r="AA17" s="17" t="n">
+      <c r="AA17" s="20" t="n">
         <v>0.2169</v>
       </c>
-      <c r="AB17" s="17" t="n">
+      <c r="AB17" s="20" t="n">
         <v>0.1941</v>
       </c>
     </row>
@@ -2027,85 +2029,85 @@
           <t>Gross Revenue Take Rate</t>
         </is>
       </c>
-      <c r="B18" s="17" t="n">
+      <c r="B18" s="20" t="n">
         <v>0.04759943521033963</v>
       </c>
-      <c r="C18" s="17" t="n">
+      <c r="C18" s="20" t="n">
         <v>0.05143855552596128</v>
       </c>
-      <c r="D18" s="17" t="n">
+      <c r="D18" s="20" t="n">
         <v>0.04795344289567624</v>
       </c>
-      <c r="E18" s="17" t="n">
+      <c r="E18" s="20" t="n">
         <v>0.0513</v>
       </c>
-      <c r="F18" s="17" t="n">
+      <c r="F18" s="20" t="n">
         <v>0.0534</v>
       </c>
-      <c r="G18" s="17" t="n">
+      <c r="G18" s="20" t="n">
         <v>0.0534</v>
       </c>
-      <c r="H18" s="17" t="n">
+      <c r="H18" s="20" t="n">
         <v>0.0473</v>
       </c>
-      <c r="I18" s="17" t="n">
+      <c r="I18" s="20" t="n">
         <v>0.0474</v>
       </c>
-      <c r="J18" s="17" t="n">
+      <c r="J18" s="20" t="n">
         <v>0.05204767330125661</v>
       </c>
-      <c r="K18" s="17" t="n">
+      <c r="K18" s="20" t="n">
         <v>0.0542479201018309</v>
       </c>
-      <c r="L18" s="17" t="n">
+      <c r="L18" s="20" t="n">
         <v>0.05800146954</v>
       </c>
-      <c r="M18" s="17" t="n">
+      <c r="M18" s="20" t="n">
         <v>0.0593103448275862</v>
       </c>
-      <c r="N18" s="17" t="n">
+      <c r="N18" s="20" t="n">
         <v>0.0530378486055777</v>
       </c>
-      <c r="O18" s="17" t="n">
+      <c r="O18" s="20" t="n">
         <v>0.05634961439588689</v>
       </c>
-      <c r="P18" s="17" t="n">
+      <c r="P18" s="20" t="n">
         <v>0.05279307631785995</v>
       </c>
-      <c r="Q18" s="17" t="n">
+      <c r="Q18" s="20" t="n">
         <v>0.05814759782070333</v>
       </c>
-      <c r="R18" s="17" t="n">
+      <c r="R18" s="20" t="n">
         <v>0.05463917525773197</v>
       </c>
-      <c r="S18" s="17" t="n">
+      <c r="S18" s="20" t="n">
         <v>0.05228758169934639</v>
       </c>
-      <c r="T18" s="17" t="n">
+      <c r="T18" s="20" t="n">
         <v>0.0473469387755102</v>
       </c>
-      <c r="U18" s="17" t="n">
+      <c r="U18" s="20" t="n">
         <v>0.04961597542242704</v>
       </c>
-      <c r="V18" s="17" t="n">
+      <c r="V18" s="20" t="n">
         <v>0.08108808290155442</v>
       </c>
-      <c r="W18" s="17" t="n">
+      <c r="W18" s="20" t="n">
         <v>0.06231231231231232</v>
       </c>
-      <c r="X18" s="17" t="n">
+      <c r="X18" s="20" t="n">
         <v>0.05742251223491028</v>
       </c>
-      <c r="Y18" s="17" t="n">
+      <c r="Y18" s="20" t="n">
         <v>0.05426862425231104</v>
       </c>
-      <c r="Z18" s="17" t="n">
+      <c r="Z18" s="20" t="n">
         <v>0.05095856816091683</v>
       </c>
-      <c r="AA18" s="17" t="n">
+      <c r="AA18" s="20" t="n">
         <v>0.05442380667066107</v>
       </c>
-      <c r="AB18" s="17" t="n">
+      <c r="AB18" s="20" t="n">
         <v>0.0523748804590373</v>
       </c>
     </row>
@@ -2115,57 +2117,57 @@
           <t>Net Revenue Take Rate</t>
         </is>
       </c>
-      <c r="B19" s="17" t="n"/>
-      <c r="C19" s="17" t="n"/>
-      <c r="D19" s="17" t="n"/>
-      <c r="E19" s="17" t="n"/>
-      <c r="F19" s="17" t="n"/>
-      <c r="G19" s="17" t="n"/>
-      <c r="H19" s="17" t="n"/>
-      <c r="I19" s="17" t="n"/>
-      <c r="J19" s="17" t="n"/>
-      <c r="K19" s="17" t="n"/>
-      <c r="L19" s="17" t="n"/>
-      <c r="M19" s="17" t="n"/>
-      <c r="N19" s="17" t="n">
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="20" t="n"/>
+      <c r="D19" s="20" t="n"/>
+      <c r="E19" s="20" t="n"/>
+      <c r="F19" s="20" t="n"/>
+      <c r="G19" s="20" t="n"/>
+      <c r="H19" s="20" t="n"/>
+      <c r="I19" s="20" t="n"/>
+      <c r="J19" s="20" t="n"/>
+      <c r="K19" s="20" t="n"/>
+      <c r="L19" s="20" t="n"/>
+      <c r="M19" s="20" t="n"/>
+      <c r="N19" s="20" t="n">
         <v>0.01596115537848606</v>
       </c>
-      <c r="O19" s="17" t="n">
+      <c r="O19" s="20" t="n">
         <v>0.02041131105398458</v>
       </c>
-      <c r="P19" s="17" t="n">
+      <c r="P19" s="20" t="n">
         <v>0.01785995279307632</v>
       </c>
-      <c r="Q19" s="17" t="n">
+      <c r="Q19" s="20" t="n">
         <v>0.01792966815255077</v>
       </c>
-      <c r="R19" s="17" t="n">
+      <c r="R19" s="20" t="n">
         <v>0.02080599812558576</v>
       </c>
-      <c r="S19" s="17" t="n">
+      <c r="S19" s="20" t="n">
         <v>0.01777777777777777</v>
       </c>
-      <c r="T19" s="17" t="n">
+      <c r="T19" s="20" t="n">
         <v>0.02102040816326531</v>
       </c>
-      <c r="U19" s="17" t="n">
+      <c r="U19" s="20" t="n">
         <v>0.02150537634408602</v>
       </c>
-      <c r="V19" s="17" t="n">
+      <c r="V19" s="20" t="n">
         <v>0.02775906735751296</v>
       </c>
-      <c r="W19" s="17" t="n">
+      <c r="W19" s="20" t="n">
         <v>0.02372372372372373</v>
       </c>
-      <c r="X19" s="17" t="n">
+      <c r="X19" s="20" t="n">
         <v>0.02137030995106036</v>
       </c>
-      <c r="Y19" s="17" t="n">
+      <c r="Y19" s="20" t="n">
         <v>0.01609570418705818</v>
       </c>
-      <c r="Z19" s="17" t="n"/>
-      <c r="AA19" s="17" t="n"/>
-      <c r="AB19" s="17" t="n"/>
+      <c r="Z19" s="20" t="n"/>
+      <c r="AA19" s="20" t="n"/>
+      <c r="AB19" s="20" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
@@ -2173,57 +2175,57 @@
           <t>Weighted Avg CoF</t>
         </is>
       </c>
-      <c r="B20" s="17" t="n"/>
-      <c r="C20" s="17" t="n"/>
-      <c r="D20" s="17" t="n"/>
-      <c r="E20" s="17" t="n"/>
-      <c r="F20" s="17" t="n"/>
-      <c r="G20" s="17" t="n"/>
-      <c r="H20" s="17" t="n"/>
-      <c r="I20" s="17" t="n"/>
-      <c r="J20" s="17" t="n"/>
-      <c r="K20" s="17" t="n"/>
-      <c r="L20" s="17" t="n"/>
-      <c r="M20" s="17" t="n"/>
-      <c r="N20" s="17" t="n">
+      <c r="B20" s="20" t="n"/>
+      <c r="C20" s="20" t="n"/>
+      <c r="D20" s="20" t="n"/>
+      <c r="E20" s="20" t="n"/>
+      <c r="F20" s="20" t="n"/>
+      <c r="G20" s="20" t="n"/>
+      <c r="H20" s="20" t="n"/>
+      <c r="I20" s="20" t="n"/>
+      <c r="J20" s="20" t="n"/>
+      <c r="K20" s="20" t="n"/>
+      <c r="L20" s="20" t="n"/>
+      <c r="M20" s="20" t="n"/>
+      <c r="N20" s="20" t="n">
         <v>0.1266</v>
       </c>
-      <c r="O20" s="17" t="n">
+      <c r="O20" s="20" t="n">
         <v>0.1293</v>
       </c>
-      <c r="P20" s="17" t="n">
+      <c r="P20" s="20" t="n">
         <v>0.1358</v>
       </c>
-      <c r="Q20" s="17" t="n">
+      <c r="Q20" s="20" t="n">
         <v>0.1334</v>
       </c>
-      <c r="R20" s="17" t="n">
+      <c r="R20" s="20" t="n">
         <v>0.136</v>
       </c>
-      <c r="S20" s="17" t="n">
+      <c r="S20" s="20" t="n">
         <v>0.146</v>
       </c>
-      <c r="T20" s="17" t="n">
+      <c r="T20" s="20" t="n">
         <v>0.1491</v>
       </c>
-      <c r="U20" s="17" t="n">
+      <c r="U20" s="20" t="n">
         <v>0.1391</v>
       </c>
-      <c r="V20" s="17" t="n">
+      <c r="V20" s="20" t="n">
         <v>0.1381</v>
       </c>
-      <c r="W20" s="17" t="n">
+      <c r="W20" s="20" t="n">
         <v>0.1375</v>
       </c>
-      <c r="X20" s="17" t="n">
+      <c r="X20" s="20" t="n">
         <v>0.1353</v>
       </c>
-      <c r="Y20" s="17" t="n">
+      <c r="Y20" s="20" t="n">
         <v>0.1345</v>
       </c>
-      <c r="Z20" s="17" t="n"/>
-      <c r="AA20" s="17" t="n"/>
-      <c r="AB20" s="17" t="n"/>
+      <c r="Z20" s="20" t="n"/>
+      <c r="AA20" s="20" t="n"/>
+      <c r="AB20" s="20" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">

</xml_diff>